<commit_message>
added new files after polishing the dir with opencode. dont know how drastic the changes wiil be but doing it anyways
</commit_message>
<xml_diff>
--- a/Excel/ABC-Marketplace-analysis.xlsx
+++ b/Excel/ABC-Marketplace-analysis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xqzme/Desktop/Data-Analyst-Portfolio/Excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{59BB159A-C799-B34C-996A-8C58622E3CCE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{751420FF-CAB0-0045-837D-CB0F95626840}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17860" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -485,7 +485,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="_-* #,##0.00\ [$₽-419]_-;\-* #,##0.00\ [$₽-419]_-;_-* &quot;-&quot;??\ [$₽-419]_-;_-@_-"/>
+    <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$₽-419]_-;\-* #,##0.00\ [$₽-419]_-;_-* &quot;-&quot;??\ [$₽-419]_-;_-@_-"/>
   </numFmts>
   <fonts count="9" x14ac:knownFonts="1">
     <font>
@@ -675,7 +675,7 @@
     </xf>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>

</xml_diff>